<commit_message>
Update the edit view so that it accurately allows for reordering, editing and existing instruction/ingredient, adding a new instruction/ingredient, or deleting on a swipe of instrutions/ingredients
</commit_message>
<xml_diff>
--- a/Project 2 Rubric Recipe App.xlsx
+++ b/Project 2 Rubric Recipe App.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/davissl_byu_edu/Documents/BYU/Fall 25/IS 543/Larson Davis Project 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{627C4493-F87C-E54A-93FC-088C44BEB1F8}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17880" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
   </bookViews>
@@ -742,6 +742,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -802,9 +826,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -831,27 +852,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1203,37 +1203,37 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="38"/>
-      <c r="E2" s="39"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
     </row>
     <row r="4" spans="2:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
     </row>
     <row r="6" spans="2:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="57"/>
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
       <c r="H6" s="16" t="s">
         <v>2</v>
       </c>
@@ -1242,97 +1242,106 @@
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B7" s="58" t="s">
+      <c r="B7" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="58"/>
-      <c r="D7" s="58"/>
-      <c r="E7" s="58"/>
-      <c r="F7" s="58"/>
-      <c r="G7" s="58"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
       <c r="H7" s="18">
         <v>2</v>
       </c>
       <c r="I7" s="6"/>
-      <c r="J7" s="19"/>
+      <c r="J7" s="19">
+        <f>SUM(H7:H26)</f>
+        <v>35</v>
+      </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="58" t="s">
+      <c r="B8" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="58"/>
-      <c r="D8" s="58"/>
-      <c r="E8" s="58"/>
-      <c r="F8" s="58"/>
-      <c r="G8" s="58"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
       <c r="H8" s="17"/>
       <c r="I8" s="21"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="58"/>
-      <c r="D9" s="58"/>
-      <c r="E9" s="58"/>
-      <c r="F9" s="58"/>
-      <c r="G9" s="58"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
       <c r="H9" s="18">
         <v>2</v>
       </c>
-      <c r="I9" s="20"/>
+      <c r="I9" s="20">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" spans="2:10" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
       <c r="H10" s="18">
         <v>4</v>
       </c>
-      <c r="I10" s="6"/>
+      <c r="I10" s="6">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B11" s="44" t="s">
+      <c r="B11" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
       <c r="H11" s="18">
         <v>2</v>
       </c>
       <c r="I11" s="6"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B12" s="44" t="s">
+      <c r="B12" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
       <c r="H12" s="18">
         <v>2</v>
       </c>
-      <c r="I12" s="6"/>
+      <c r="I12" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="44" t="s">
+      <c r="B13" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
       <c r="H13" s="18">
         <v>2</v>
       </c>
@@ -1340,14 +1349,14 @@
       <c r="J13" s="19"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B14" s="59" t="s">
+      <c r="B14" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="59"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="59"/>
-      <c r="F14" s="59"/>
-      <c r="G14" s="59"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
       <c r="H14" s="18">
         <v>2</v>
       </c>
@@ -1355,208 +1364,216 @@
       <c r="J14" s="19"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="59"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="59"/>
-      <c r="F15" s="59"/>
-      <c r="G15" s="59"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
       <c r="H15" s="18">
         <v>2</v>
       </c>
       <c r="I15" s="6"/>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B16" s="59" t="s">
+      <c r="B16" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="59"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="59"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="59"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
       <c r="H16" s="18">
         <v>2</v>
       </c>
-      <c r="I16" s="22"/>
+      <c r="I16" s="22">
+        <v>2</v>
+      </c>
       <c r="J16" s="19"/>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B17" s="59" t="s">
+      <c r="B17" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
       <c r="H17" s="18">
         <v>2</v>
       </c>
       <c r="I17" s="8"/>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B18" s="59" t="s">
+      <c r="B18" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="59"/>
-      <c r="D18" s="59"/>
-      <c r="E18" s="59"/>
-      <c r="F18" s="59"/>
-      <c r="G18" s="59"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
       <c r="H18" s="18">
         <v>2</v>
       </c>
       <c r="I18" s="6"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="60"/>
-      <c r="D19" s="60"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="60"/>
-      <c r="G19" s="60"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
       <c r="H19" s="10">
         <v>2</v>
       </c>
-      <c r="I19" s="8"/>
+      <c r="I19" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="59"/>
-      <c r="D20" s="59"/>
-      <c r="E20" s="59"/>
-      <c r="F20" s="59"/>
-      <c r="G20" s="59"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
       <c r="H20" s="9">
         <v>2</v>
       </c>
-      <c r="I20" s="6"/>
+      <c r="I20" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B21" s="59" t="s">
+      <c r="B21" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="59"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
       <c r="H21" s="9">
         <v>2</v>
       </c>
-      <c r="I21" s="6"/>
+      <c r="I21" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B22" s="54" t="s">
+      <c r="B22" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="55"/>
-      <c r="D22" s="55"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="55"/>
-      <c r="G22" s="56"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="27"/>
       <c r="H22" s="9">
         <v>1</v>
       </c>
       <c r="I22" s="6"/>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B23" s="54" t="s">
+      <c r="B23" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="55"/>
-      <c r="D23" s="55"/>
-      <c r="E23" s="55"/>
-      <c r="F23" s="55"/>
-      <c r="G23" s="56"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="27"/>
       <c r="H23" s="9">
         <v>1</v>
       </c>
       <c r="I23" s="6"/>
     </row>
     <row r="24" spans="2:10" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="54" t="s">
+      <c r="B24" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="55"/>
-      <c r="G24" s="56"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="27"/>
       <c r="H24" s="9">
         <v>1</v>
       </c>
       <c r="I24" s="6"/>
     </row>
     <row r="25" spans="2:10" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="48" t="s">
+      <c r="B25" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="50"/>
+      <c r="C25" s="56"/>
+      <c r="D25" s="56"/>
+      <c r="E25" s="56"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="57"/>
       <c r="H25" s="4">
         <v>1</v>
       </c>
       <c r="I25" s="5"/>
     </row>
     <row r="26" spans="2:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="51" t="s">
+      <c r="B26" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="53"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="60"/>
       <c r="H26" s="4">
         <v>1</v>
       </c>
       <c r="I26" s="5"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B27" s="45" t="s">
+      <c r="B27" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="46"/>
-      <c r="D27" s="46"/>
-      <c r="E27" s="46"/>
-      <c r="F27" s="46"/>
-      <c r="G27" s="47"/>
+      <c r="C27" s="53"/>
+      <c r="D27" s="53"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="53"/>
+      <c r="G27" s="54"/>
       <c r="H27" s="7" t="s">
         <v>10</v>
       </c>
       <c r="I27" s="8"/>
     </row>
     <row r="28" spans="2:10" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="34"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="36"/>
+      <c r="B28" s="42"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="43"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="44"/>
       <c r="H28" s="12"/>
       <c r="I28" s="11"/>
       <c r="J28" s="3"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="40"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
-      <c r="G29" s="43"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="48"/>
+      <c r="G29" s="51"/>
       <c r="H29" s="7" t="s">
         <v>5</v>
       </c>
@@ -1566,12 +1583,12 @@
       </c>
     </row>
     <row r="30" spans="2:10" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="34"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
-      <c r="G30" s="36"/>
+      <c r="B30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="44"/>
       <c r="H30" s="13"/>
       <c r="I30" s="11"/>
       <c r="J30" s="3"/>
@@ -1586,7 +1603,7 @@
       </c>
       <c r="I31" s="1">
         <f>SUM(I7:I30)</f>
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.2">
@@ -1595,143 +1612,160 @@
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="24" t="s">
+      <c r="B33" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="24"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
     </row>
     <row r="35" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="24" t="s">
+      <c r="B35" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="24"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
+      <c r="I35" s="32"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="25"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="27"/>
+      <c r="B36" s="33"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="34"/>
+      <c r="I36" s="35"/>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B37" s="28"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="29"/>
-      <c r="H37" s="29"/>
-      <c r="I37" s="30"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
+      <c r="G37" s="37"/>
+      <c r="H37" s="37"/>
+      <c r="I37" s="38"/>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B38" s="28"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="30"/>
+      <c r="B38" s="36"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="37"/>
+      <c r="E38" s="37"/>
+      <c r="F38" s="37"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="37"/>
+      <c r="I38" s="38"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B39" s="28"/>
-      <c r="C39" s="29"/>
-      <c r="D39" s="29"/>
-      <c r="E39" s="29"/>
-      <c r="F39" s="29"/>
-      <c r="G39" s="29"/>
-      <c r="H39" s="29"/>
-      <c r="I39" s="30"/>
+      <c r="B39" s="36"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="37"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="37"/>
+      <c r="I39" s="38"/>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B40" s="31"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
-      <c r="H40" s="32"/>
-      <c r="I40" s="33"/>
+      <c r="B40" s="39"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="40"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="41"/>
     </row>
     <row r="42" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="24" t="s">
+      <c r="B42" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C42" s="24"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
-      <c r="G42" s="24"/>
-      <c r="H42" s="24"/>
-      <c r="I42" s="24"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="32"/>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B43" s="25"/>
-      <c r="C43" s="26"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="26"/>
-      <c r="G43" s="26"/>
-      <c r="H43" s="26"/>
-      <c r="I43" s="27"/>
+      <c r="B43" s="33"/>
+      <c r="C43" s="34"/>
+      <c r="D43" s="34"/>
+      <c r="E43" s="34"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="34"/>
+      <c r="H43" s="34"/>
+      <c r="I43" s="35"/>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B44" s="28"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="29"/>
-      <c r="E44" s="29"/>
-      <c r="F44" s="29"/>
-      <c r="G44" s="29"/>
-      <c r="H44" s="29"/>
-      <c r="I44" s="30"/>
+      <c r="B44" s="36"/>
+      <c r="C44" s="37"/>
+      <c r="D44" s="37"/>
+      <c r="E44" s="37"/>
+      <c r="F44" s="37"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="37"/>
+      <c r="I44" s="38"/>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B45" s="28"/>
-      <c r="C45" s="29"/>
-      <c r="D45" s="29"/>
-      <c r="E45" s="29"/>
-      <c r="F45" s="29"/>
-      <c r="G45" s="29"/>
-      <c r="H45" s="29"/>
-      <c r="I45" s="30"/>
+      <c r="B45" s="36"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="37"/>
+      <c r="F45" s="37"/>
+      <c r="G45" s="37"/>
+      <c r="H45" s="37"/>
+      <c r="I45" s="38"/>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B46" s="28"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="29"/>
-      <c r="E46" s="29"/>
-      <c r="F46" s="29"/>
-      <c r="G46" s="29"/>
-      <c r="H46" s="29"/>
-      <c r="I46" s="30"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="37"/>
+      <c r="I46" s="38"/>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B47" s="31"/>
-      <c r="C47" s="32"/>
-      <c r="D47" s="32"/>
-      <c r="E47" s="32"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
-      <c r="H47" s="32"/>
-      <c r="I47" s="33"/>
+      <c r="B47" s="39"/>
+      <c r="C47" s="40"/>
+      <c r="D47" s="40"/>
+      <c r="E47" s="40"/>
+      <c r="F47" s="40"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="40"/>
+      <c r="I47" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B43:I47"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B36:I40"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B26:G26"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B23:G23"/>
     <mergeCell ref="B24:G24"/>
@@ -1748,23 +1782,6 @@
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="B17:G17"/>
     <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B43:I47"/>
-    <mergeCell ref="B30:G30"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B36:I40"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="B22:G22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
categories are new working as desired, they can be created, edited, and deleted
</commit_message>
<xml_diff>
--- a/Project 2 Rubric Recipe App.xlsx
+++ b/Project 2 Rubric Recipe App.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/davissl_byu_edu/Documents/BYU/Fall 25/IS 543/Larson Davis Project 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{627C4493-F87C-E54A-93FC-088C44BEB1F8}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77986696-9A2F-294E-87B3-E820428D6707}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17880" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
   <si>
     <t>Name:</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>Davis Larson</t>
+  </si>
+  <si>
+    <t>?</t>
   </si>
 </sst>
 </file>
@@ -1315,7 +1318,9 @@
       <c r="H11" s="18">
         <v>2</v>
       </c>
-      <c r="I11" s="6"/>
+      <c r="I11" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B12" s="30" t="s">
@@ -1345,7 +1350,9 @@
       <c r="H13" s="18">
         <v>2</v>
       </c>
-      <c r="I13" s="23"/>
+      <c r="I13" s="23">
+        <v>2</v>
+      </c>
       <c r="J13" s="19"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
@@ -1360,7 +1367,9 @@
       <c r="H14" s="18">
         <v>2</v>
       </c>
-      <c r="I14" s="6"/>
+      <c r="I14" s="6">
+        <v>2</v>
+      </c>
       <c r="J14" s="19"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
@@ -1375,7 +1384,12 @@
       <c r="H15" s="18">
         <v>2</v>
       </c>
-      <c r="I15" s="6"/>
+      <c r="I15" s="6">
+        <v>2</v>
+      </c>
+      <c r="J15" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B16" s="24" t="s">
@@ -1406,7 +1420,9 @@
       <c r="H17" s="18">
         <v>2</v>
       </c>
-      <c r="I17" s="8"/>
+      <c r="I17" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B18" s="24" t="s">
@@ -1420,7 +1436,12 @@
       <c r="H18" s="18">
         <v>2</v>
       </c>
-      <c r="I18" s="6"/>
+      <c r="I18" s="6">
+        <v>2</v>
+      </c>
+      <c r="J18" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B19" s="31" t="s">
@@ -1482,7 +1503,9 @@
       <c r="H22" s="9">
         <v>1</v>
       </c>
-      <c r="I22" s="6"/>
+      <c r="I22" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B23" s="25" t="s">
@@ -1496,7 +1519,9 @@
       <c r="H23" s="9">
         <v>1</v>
       </c>
-      <c r="I23" s="6"/>
+      <c r="I23" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="24" spans="2:10" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B24" s="25" t="s">
@@ -1603,7 +1628,7 @@
       </c>
       <c r="I31" s="1">
         <f>SUM(I7:I30)</f>
-        <v>16</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
add a new recipe and make default landing page the allRecipes page
</commit_message>
<xml_diff>
--- a/Project 2 Rubric Recipe App.xlsx
+++ b/Project 2 Rubric Recipe App.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/davissl_byu_edu/Documents/BYU/Fall 25/IS 543/Larson Davis Project 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77986696-9A2F-294E-87B3-E820428D6707}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{805A1A12-356E-8241-A082-21B22EE74246}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Name:</t>
   </si>
@@ -1387,9 +1387,6 @@
       <c r="I15" s="6">
         <v>2</v>
       </c>
-      <c r="J15" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B16" s="24" t="s">

</xml_diff>

<commit_message>
spelling correction and color unification
</commit_message>
<xml_diff>
--- a/Project 2 Rubric Recipe App.xlsx
+++ b/Project 2 Rubric Recipe App.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/davissl_byu_edu/Documents/BYU/Fall 25/IS 543/Larson Davis Project 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{805A1A12-356E-8241-A082-21B22EE74246}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B40EF72F-B2E8-D940-A1B3-CCBCBC4436A3}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Name:</t>
   </si>
@@ -147,7 +147,13 @@
     <t>Davis Larson</t>
   </si>
   <si>
-    <t>?</t>
+    <t>searching by difficulty is not working right</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>check on this</t>
   </si>
 </sst>
 </file>
@@ -686,7 +692,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -745,116 +750,119 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -871,6 +879,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1206,576 +1218,596 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="45" t="s">
+      <c r="C2" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="42"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
     </row>
     <row r="4" spans="2:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
     </row>
     <row r="6" spans="2:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="I6" s="16" t="s">
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="I6" s="15" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="18">
-        <v>2</v>
-      </c>
-      <c r="I7" s="6"/>
-      <c r="J7" s="19">
+      <c r="C7" s="59"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
+      <c r="H7" s="17">
+        <v>2</v>
+      </c>
+      <c r="I7" s="5">
+        <v>2</v>
+      </c>
+      <c r="J7" s="18">
         <f>SUM(H7:H26)</f>
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="21"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="18">
-        <v>2</v>
-      </c>
-      <c r="I9" s="20">
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="17">
+        <v>2</v>
+      </c>
+      <c r="I9" s="19">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="2:10" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="18">
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="17">
         <v>4</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="5">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="18">
-        <v>2</v>
-      </c>
-      <c r="I11" s="6">
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="17">
+        <v>2</v>
+      </c>
+      <c r="I11" s="5">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="18">
-        <v>2</v>
-      </c>
-      <c r="I12" s="6">
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="17">
+        <v>2</v>
+      </c>
+      <c r="I12" s="5">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="18">
-        <v>2</v>
-      </c>
-      <c r="I13" s="23">
-        <v>2</v>
-      </c>
-      <c r="J13" s="19"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="47"/>
+      <c r="G13" s="47"/>
+      <c r="H13" s="17">
+        <v>2</v>
+      </c>
+      <c r="I13" s="22">
+        <v>2</v>
+      </c>
+      <c r="J13" s="18"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="18">
-        <v>2</v>
-      </c>
-      <c r="I14" s="6">
-        <v>2</v>
-      </c>
-      <c r="J14" s="19"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="17">
+        <v>2</v>
+      </c>
+      <c r="I14" s="5">
+        <v>2</v>
+      </c>
+      <c r="J14" s="18"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="18">
-        <v>2</v>
-      </c>
-      <c r="I15" s="6">
+      <c r="C15" s="57"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="57"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="17">
+        <v>2</v>
+      </c>
+      <c r="I15" s="5">
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="18">
-        <v>2</v>
-      </c>
-      <c r="I16" s="22">
-        <v>2</v>
-      </c>
-      <c r="J16" s="19"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="57"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="17">
+        <v>2</v>
+      </c>
+      <c r="I16" s="21">
+        <v>2</v>
+      </c>
+      <c r="J16" s="18"/>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="18">
-        <v>2</v>
-      </c>
-      <c r="I17" s="8">
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="17">
+        <v>2</v>
+      </c>
+      <c r="I17" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="57" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="18">
-        <v>2</v>
-      </c>
-      <c r="I18" s="6">
+      <c r="C18" s="57"/>
+      <c r="D18" s="57"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="17">
+        <v>2</v>
+      </c>
+      <c r="I18" s="5">
         <v>2</v>
       </c>
       <c r="J18" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="10">
-        <v>2</v>
-      </c>
-      <c r="I19" s="8">
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="9">
+        <v>2</v>
+      </c>
+      <c r="I19" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="9">
-        <v>2</v>
-      </c>
-      <c r="I20" s="6">
+      <c r="C20" s="57"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="57"/>
+      <c r="H20" s="8">
+        <v>2</v>
+      </c>
+      <c r="I20" s="5">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="9">
-        <v>2</v>
-      </c>
-      <c r="I21" s="6">
+      <c r="C21" s="57"/>
+      <c r="D21" s="57"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="8">
+        <v>2</v>
+      </c>
+      <c r="I21" s="5">
         <v>2</v>
       </c>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="9">
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="8">
         <v>1</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B23" s="25" t="s">
+      <c r="B23" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="9">
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="8">
         <v>1</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="2:10" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="25" t="s">
+      <c r="B24" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="9">
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="8">
         <v>1</v>
       </c>
-      <c r="I24" s="6"/>
+      <c r="I24" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" spans="2:10" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="55" t="s">
+      <c r="B25" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="56"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="4">
+      <c r="C25" s="52"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="53"/>
+      <c r="H25" s="3">
         <v>1</v>
       </c>
-      <c r="I25" s="5"/>
+      <c r="I25" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="26" spans="2:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="58" t="s">
+      <c r="B26" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="60"/>
-      <c r="H26" s="4">
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="55"/>
+      <c r="F26" s="55"/>
+      <c r="G26" s="56"/>
+      <c r="H26" s="3">
         <v>1</v>
       </c>
-      <c r="I26" s="5"/>
+      <c r="I26" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B27" s="52" t="s">
+      <c r="B27" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="53"/>
-      <c r="G27" s="54"/>
-      <c r="H27" s="7" t="s">
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="50"/>
+      <c r="H27" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I27" s="8"/>
+      <c r="I27" s="7">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="2:10" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="42"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="3"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="10"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B29" s="50" t="s">
+      <c r="B29" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="51"/>
-      <c r="H29" s="7" t="s">
+      <c r="C29" s="43"/>
+      <c r="D29" s="43"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="43"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I29" s="8"/>
+      <c r="I29" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="J29" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="30" spans="2:10" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="42"/>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="3"/>
+      <c r="B30" s="37"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="60" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="G31" s="14" t="s">
+      <c r="G31" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="15" t="str">
+      <c r="H31" s="14" t="str">
         <f>"≤ "&amp;SUM(H7:H26)</f>
         <v>≤ 35</v>
       </c>
       <c r="I31" s="1">
         <f>SUM(I7:I30)</f>
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="G32" s="14"/>
-      <c r="H32" s="15"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="14"/>
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27"/>
     </row>
     <row r="35" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="32" t="s">
+      <c r="B35" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="32"/>
-      <c r="I35" s="32"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="33"/>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="34"/>
-      <c r="F36" s="34"/>
-      <c r="G36" s="34"/>
-      <c r="H36" s="34"/>
-      <c r="I36" s="35"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="30"/>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B37" s="36"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="37"/>
-      <c r="I37" s="38"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="33"/>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B38" s="36"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="37"/>
-      <c r="F38" s="37"/>
-      <c r="G38" s="37"/>
-      <c r="H38" s="37"/>
-      <c r="I38" s="38"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="33"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B39" s="36"/>
-      <c r="C39" s="37"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="37"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="37"/>
-      <c r="H39" s="37"/>
-      <c r="I39" s="38"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="33"/>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B40" s="39"/>
-      <c r="C40" s="40"/>
-      <c r="D40" s="40"/>
-      <c r="E40" s="40"/>
-      <c r="F40" s="40"/>
-      <c r="G40" s="40"/>
-      <c r="H40" s="40"/>
-      <c r="I40" s="41"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="35"/>
+      <c r="E40" s="35"/>
+      <c r="F40" s="35"/>
+      <c r="G40" s="35"/>
+      <c r="H40" s="35"/>
+      <c r="I40" s="36"/>
     </row>
     <row r="42" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="32" t="s">
+      <c r="B42" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="32"/>
+      <c r="C42" s="27"/>
+      <c r="D42" s="27"/>
+      <c r="E42" s="27"/>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="27"/>
+      <c r="I42" s="27"/>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B43" s="33"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="35"/>
+      <c r="B43" s="28"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="30"/>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B44" s="36"/>
-      <c r="C44" s="37"/>
-      <c r="D44" s="37"/>
-      <c r="E44" s="37"/>
-      <c r="F44" s="37"/>
-      <c r="G44" s="37"/>
-      <c r="H44" s="37"/>
-      <c r="I44" s="38"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="33"/>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B45" s="36"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="37"/>
-      <c r="F45" s="37"/>
-      <c r="G45" s="37"/>
-      <c r="H45" s="37"/>
-      <c r="I45" s="38"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="32"/>
+      <c r="H45" s="32"/>
+      <c r="I45" s="33"/>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B46" s="36"/>
-      <c r="C46" s="37"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="37"/>
-      <c r="F46" s="37"/>
-      <c r="G46" s="37"/>
-      <c r="H46" s="37"/>
-      <c r="I46" s="38"/>
+      <c r="B46" s="31"/>
+      <c r="C46" s="32"/>
+      <c r="D46" s="32"/>
+      <c r="E46" s="32"/>
+      <c r="F46" s="32"/>
+      <c r="G46" s="32"/>
+      <c r="H46" s="32"/>
+      <c r="I46" s="33"/>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B47" s="39"/>
-      <c r="C47" s="40"/>
-      <c r="D47" s="40"/>
-      <c r="E47" s="40"/>
-      <c r="F47" s="40"/>
-      <c r="G47" s="40"/>
-      <c r="H47" s="40"/>
-      <c r="I47" s="41"/>
+      <c r="B47" s="34"/>
+      <c r="C47" s="35"/>
+      <c r="D47" s="35"/>
+      <c r="E47" s="35"/>
+      <c r="F47" s="35"/>
+      <c r="G47" s="35"/>
+      <c r="H47" s="35"/>
+      <c r="I47" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B43:I47"/>
-    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B18:G18"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="B4:I4"/>
@@ -1792,18 +1824,11 @@
     <mergeCell ref="B23:G23"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B14:G14"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B43:I47"/>
+    <mergeCell ref="B30:G30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
use the .searchable provided by the NavigationSplitView
</commit_message>
<xml_diff>
--- a/Project 2 Rubric Recipe App.xlsx
+++ b/Project 2 Rubric Recipe App.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/davissl_byu_edu/Documents/BYU/Fall 25/IS 543/Larson Davis Project 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B40EF72F-B2E8-D940-A1B3-CCBCBC4436A3}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8148F704-9B78-4741-BD39-1CB23FF5B395}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
   </bookViews>
@@ -147,13 +147,13 @@
     <t>Davis Larson</t>
   </si>
   <si>
-    <t>searching by difficulty is not working right</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
-    <t>check on this</t>
+    <t>I tried to add searching by difficulty but was having issues. After some reasearch I learned that there were some limitations with using #Prediecate in the  FetchDescriptorand an enum to filter. I decided to take it out because it was taking too much time but it seemed like a simple thing but for the life of me I couldn't get it to work. Another issue that I was having a little difficulty with was handling editing mode in all the nested views. In the category list view there is certain way to edit the categories (by swiping on the category).I was having trouble making the edit button (like the one I have on the RecipeListView) give an option to edit, or make it so that when a user is in edit mode it brings up the edit view. I was getting the nested views mixed up and it was making it hard to get the UI to move to editing like I wanted. I got it to work but I would say that it is not as understandable as it could be getting to editing views of the reciepes or categories. I think after a little bit of time using the app it becomes understandable but it is not super clear up front.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I enjoyed this project. It was even an app that is useful and practical for my life. It was also cool to see how much swiftUI pre builds stuff for development. I also think I had a greater understanding of what I was writing for this project. I think project 1 I was flying by the seat of my pants but this one I was able to understand with much more clarity how things connected. The animals swift example was super helpful for me too. I think having projects like that that we study in class or on our own is super helpful. I think it was hard for me to find valuable questions to ask in a classroom setting. I appriciated the time that was given to ask questions in class but I don't feel that my questions were easy to ask or answer in a classroom setting. AI was great at answering most of these questions. I feel like repalcing some of that QnA time in class with demos of a technique or aspect of the project would have been much more benificial. </t>
   </si>
 </sst>
 </file>
@@ -686,7 +686,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -750,6 +750,105 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -759,110 +858,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1202,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEAB4736-463A-B544-BE22-2FA081663951}">
-  <dimension ref="B1:J47"/>
+  <dimension ref="B1:J48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="0.83203125" customWidth="1"/>
@@ -1218,37 +1221,37 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="41"/>
-      <c r="E2" s="42"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="29"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
     </row>
     <row r="4" spans="2:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
     </row>
     <row r="6" spans="2:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="58" t="s">
+      <c r="B6" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
-      <c r="G6" s="58"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
       <c r="H6" s="15" t="s">
         <v>2</v>
       </c>
@@ -1257,14 +1260,14 @@
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B7" s="59" t="s">
+      <c r="B7" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="59"/>
-      <c r="D7" s="59"/>
-      <c r="E7" s="59"/>
-      <c r="F7" s="59"/>
-      <c r="G7" s="59"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
       <c r="H7" s="17">
         <v>2</v>
       </c>
@@ -1277,26 +1280,26 @@
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="59" t="s">
+      <c r="B8" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="59"/>
-      <c r="D8" s="59"/>
-      <c r="E8" s="59"/>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
       <c r="H8" s="16"/>
       <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B9" s="59" t="s">
+      <c r="B9" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
       <c r="H9" s="17">
         <v>2</v>
       </c>
@@ -1305,14 +1308,14 @@
       </c>
     </row>
     <row r="10" spans="2:10" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="47" t="s">
+      <c r="B10" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
       <c r="H10" s="17">
         <v>4</v>
       </c>
@@ -1321,14 +1324,14 @@
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
       <c r="H11" s="17">
         <v>2</v>
       </c>
@@ -1337,14 +1340,14 @@
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B12" s="47" t="s">
+      <c r="B12" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
       <c r="H12" s="17">
         <v>2</v>
       </c>
@@ -1353,14 +1356,14 @@
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="47" t="s">
+      <c r="B13" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="47"/>
-      <c r="D13" s="47"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="47"/>
-      <c r="G13" s="47"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
       <c r="H13" s="17">
         <v>2</v>
       </c>
@@ -1370,14 +1373,14 @@
       <c r="J13" s="18"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B14" s="57" t="s">
+      <c r="B14" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="57"/>
-      <c r="G14" s="57"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
       <c r="H14" s="17">
         <v>2</v>
       </c>
@@ -1387,14 +1390,14 @@
       <c r="J14" s="18"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B15" s="57" t="s">
+      <c r="B15" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="57"/>
-      <c r="G15" s="57"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
       <c r="H15" s="17">
         <v>2</v>
       </c>
@@ -1403,14 +1406,14 @@
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B16" s="57" t="s">
+      <c r="B16" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="57"/>
-      <c r="D16" s="57"/>
-      <c r="E16" s="57"/>
-      <c r="F16" s="57"/>
-      <c r="G16" s="57"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
       <c r="H16" s="17">
         <v>2</v>
       </c>
@@ -1420,14 +1423,14 @@
       <c r="J16" s="18"/>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B17" s="57" t="s">
+      <c r="B17" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="57"/>
-      <c r="D17" s="57"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
       <c r="H17" s="17">
         <v>2</v>
       </c>
@@ -1436,33 +1439,30 @@
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B18" s="57" t="s">
+      <c r="B18" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="57"/>
-      <c r="F18" s="57"/>
-      <c r="G18" s="57"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
       <c r="H18" s="17">
         <v>2</v>
       </c>
       <c r="I18" s="5">
         <v>2</v>
       </c>
-      <c r="J18" t="s">
-        <v>37</v>
-      </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
+      <c r="C19" s="60"/>
+      <c r="D19" s="60"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="60"/>
+      <c r="G19" s="60"/>
       <c r="H19" s="9">
         <v>2</v>
       </c>
@@ -1471,14 +1471,14 @@
       </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B20" s="57" t="s">
+      <c r="B20" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
       <c r="H20" s="8">
         <v>2</v>
       </c>
@@ -1487,14 +1487,14 @@
       </c>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B21" s="57" t="s">
+      <c r="B21" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="57"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="57"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
       <c r="H21" s="8">
         <v>2</v>
       </c>
@@ -1503,14 +1503,14 @@
       </c>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="25"/>
+      <c r="C22" s="57"/>
+      <c r="D22" s="57"/>
+      <c r="E22" s="57"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="58"/>
       <c r="H22" s="8">
         <v>1</v>
       </c>
@@ -1519,14 +1519,14 @@
       </c>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="25"/>
+      <c r="C23" s="57"/>
+      <c r="D23" s="57"/>
+      <c r="E23" s="57"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="58"/>
       <c r="H23" s="8">
         <v>1</v>
       </c>
@@ -1535,14 +1535,14 @@
       </c>
     </row>
     <row r="24" spans="2:10" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="25"/>
+      <c r="C24" s="57"/>
+      <c r="D24" s="57"/>
+      <c r="E24" s="57"/>
+      <c r="F24" s="57"/>
+      <c r="G24" s="58"/>
       <c r="H24" s="8">
         <v>1</v>
       </c>
@@ -1551,14 +1551,14 @@
       </c>
     </row>
     <row r="25" spans="2:10" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="51" t="s">
+      <c r="B25" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="52"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="52"/>
-      <c r="F25" s="52"/>
-      <c r="G25" s="53"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="51"/>
+      <c r="E25" s="51"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="52"/>
       <c r="H25" s="3">
         <v>1</v>
       </c>
@@ -1567,14 +1567,14 @@
       </c>
     </row>
     <row r="26" spans="2:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="55"/>
-      <c r="D26" s="55"/>
-      <c r="E26" s="55"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="56"/>
+      <c r="C26" s="54"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="55"/>
       <c r="H26" s="3">
         <v>1</v>
       </c>
@@ -1583,14 +1583,14 @@
       </c>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B27" s="48" t="s">
+      <c r="B27" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="49"/>
-      <c r="D27" s="49"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="50"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="G27" s="49"/>
       <c r="H27" s="6" t="s">
         <v>10</v>
       </c>
@@ -1599,46 +1599,44 @@
       </c>
     </row>
     <row r="28" spans="2:10" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="37"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="39"/>
+      <c r="B28" s="44"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="45"/>
+      <c r="G28" s="46"/>
       <c r="H28" s="11"/>
       <c r="I28" s="10"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B29" s="45" t="s">
+      <c r="B29" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="43"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="46"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="43"/>
       <c r="H29" s="6" t="s">
         <v>5</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J29" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="30" spans="2:10" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="37"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="39"/>
+      <c r="B30" s="44"/>
+      <c r="C30" s="45"/>
+      <c r="D30" s="45"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="45"/>
+      <c r="G30" s="46"/>
       <c r="H30" s="12"/>
       <c r="I30" s="10"/>
-      <c r="J30" s="60" t="s">
-        <v>35</v>
-      </c>
+      <c r="J30" s="23"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G31" s="13" t="s">
@@ -1659,155 +1657,162 @@
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="27" t="s">
+      <c r="B33" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="27"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="27"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
     </row>
     <row r="35" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="27" t="s">
+      <c r="B35" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="27"/>
-      <c r="I35" s="27"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
+      <c r="I35" s="32"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="28"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="29"/>
-      <c r="F36" s="29"/>
-      <c r="G36" s="29"/>
-      <c r="H36" s="29"/>
-      <c r="I36" s="30"/>
+      <c r="B36" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="34"/>
+      <c r="I36" s="35"/>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B37" s="31"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="33"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
+      <c r="G37" s="37"/>
+      <c r="H37" s="37"/>
+      <c r="I37" s="38"/>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B38" s="31"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="32"/>
-      <c r="I38" s="33"/>
+      <c r="B38" s="36"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="37"/>
+      <c r="E38" s="37"/>
+      <c r="F38" s="37"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="37"/>
+      <c r="I38" s="38"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B39" s="31"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="33"/>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B40" s="34"/>
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="35"/>
-      <c r="H40" s="35"/>
-      <c r="I40" s="36"/>
-    </row>
-    <row r="42" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="27" t="s">
+      <c r="B39" s="36"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="37"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="37"/>
+      <c r="I39" s="38"/>
+    </row>
+    <row r="40" spans="2:9" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B40" s="39"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="40"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="41"/>
+    </row>
+    <row r="41" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B41" s="61"/>
+      <c r="C41" s="61"/>
+      <c r="D41" s="61"/>
+      <c r="E41" s="61"/>
+      <c r="F41" s="61"/>
+      <c r="G41" s="61"/>
+      <c r="H41" s="61"/>
+      <c r="I41" s="61"/>
+    </row>
+    <row r="43" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B43" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C42" s="27"/>
-      <c r="D42" s="27"/>
-      <c r="E42" s="27"/>
-      <c r="F42" s="27"/>
-      <c r="G42" s="27"/>
-      <c r="H42" s="27"/>
-      <c r="I42" s="27"/>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B43" s="28"/>
-      <c r="C43" s="29"/>
-      <c r="D43" s="29"/>
-      <c r="E43" s="29"/>
-      <c r="F43" s="29"/>
-      <c r="G43" s="29"/>
-      <c r="H43" s="29"/>
-      <c r="I43" s="30"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="32"/>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B44" s="31"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="33"/>
+      <c r="B44" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="C44" s="34"/>
+      <c r="D44" s="34"/>
+      <c r="E44" s="34"/>
+      <c r="F44" s="34"/>
+      <c r="G44" s="34"/>
+      <c r="H44" s="34"/>
+      <c r="I44" s="35"/>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B45" s="31"/>
-      <c r="C45" s="32"/>
-      <c r="D45" s="32"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="32"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="33"/>
+      <c r="B45" s="36"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="37"/>
+      <c r="F45" s="37"/>
+      <c r="G45" s="37"/>
+      <c r="H45" s="37"/>
+      <c r="I45" s="38"/>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B46" s="31"/>
-      <c r="C46" s="32"/>
-      <c r="D46" s="32"/>
-      <c r="E46" s="32"/>
-      <c r="F46" s="32"/>
-      <c r="G46" s="32"/>
-      <c r="H46" s="32"/>
-      <c r="I46" s="33"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="37"/>
+      <c r="I46" s="38"/>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B47" s="34"/>
-      <c r="C47" s="35"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="35"/>
-      <c r="F47" s="35"/>
-      <c r="G47" s="35"/>
-      <c r="H47" s="35"/>
-      <c r="I47" s="36"/>
+      <c r="B47" s="36"/>
+      <c r="C47" s="37"/>
+      <c r="D47" s="37"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="37"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="37"/>
+      <c r="I47" s="38"/>
+    </row>
+    <row r="48" spans="2:9" ht="117" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B48" s="39"/>
+      <c r="C48" s="40"/>
+      <c r="D48" s="40"/>
+      <c r="E48" s="40"/>
+      <c r="F48" s="40"/>
+      <c r="G48" s="40"/>
+      <c r="H48" s="40"/>
+      <c r="I48" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B14:G14"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B44:I48"/>
+    <mergeCell ref="B30:G30"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="B4:I4"/>
@@ -1824,11 +1829,18 @@
     <mergeCell ref="B23:G23"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B43:I47"/>
-    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B18:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
update the readme a little bit
</commit_message>
<xml_diff>
--- a/Project 2 Rubric Recipe App.xlsx
+++ b/Project 2 Rubric Recipe App.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/davissl_byu_edu/Documents/BYU/Fall 25/IS 543/Larson Davis Project 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8148F704-9B78-4741-BD39-1CB23FF5B395}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBA1693D-5A96-B044-8F1E-CB661F555780}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
+    <workbookView xWindow="32600" yWindow="-9340" windowWidth="30240" windowHeight="17680" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -150,10 +150,10 @@
     <t>N</t>
   </si>
   <si>
-    <t>I tried to add searching by difficulty but was having issues. After some reasearch I learned that there were some limitations with using #Prediecate in the  FetchDescriptorand an enum to filter. I decided to take it out because it was taking too much time but it seemed like a simple thing but for the life of me I couldn't get it to work. Another issue that I was having a little difficulty with was handling editing mode in all the nested views. In the category list view there is certain way to edit the categories (by swiping on the category).I was having trouble making the edit button (like the one I have on the RecipeListView) give an option to edit, or make it so that when a user is in edit mode it brings up the edit view. I was getting the nested views mixed up and it was making it hard to get the UI to move to editing like I wanted. I got it to work but I would say that it is not as understandable as it could be getting to editing views of the reciepes or categories. I think after a little bit of time using the app it becomes understandable but it is not super clear up front.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I enjoyed this project. It was even an app that is useful and practical for my life. It was also cool to see how much swiftUI pre builds stuff for development. I also think I had a greater understanding of what I was writing for this project. I think project 1 I was flying by the seat of my pants but this one I was able to understand with much more clarity how things connected. The animals swift example was super helpful for me too. I think having projects like that that we study in class or on our own is super helpful. I think it was hard for me to find valuable questions to ask in a classroom setting. I appriciated the time that was given to ask questions in class but I don't feel that my questions were easy to ask or answer in a classroom setting. AI was great at answering most of these questions. I feel like repalcing some of that QnA time in class with demos of a technique or aspect of the project would have been much more benificial. </t>
+    <t>I tried to add searching by difficulty level but was having issues. After some reasearch I learned that there were some limitations with using #Prediecate in the  FetchDescriptorand an enum to filter. I decided to take it out because it wasn't a requirement and it was taking too much time but it seemed like a simple thing but for the life of me I couldn't get it to work. Another issue that I was having a little difficulty with was handling editing mode in all the nested views. In the category list view there is certain way to edit the categories (by swiping on the category).I was having trouble making the built in edit button give an option to edit the recipe, or make it so that when a user is in edit mode it brings up the edit view when they tap on the recipe. I was getting the nested views mixed up and it was making it hard to get the UI to move to editing like I wanted. I got it to work by removing the edit button itself and add a swipe action but I would say that it is not as understandable as it could be getting to editing views of the reciepes or categories. I think after a little bit of time using the app it becomes understandable but it is not super clear up front.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I enjoyed this project. It was even an app that is useful and practical for my life. It was also cool to see how much swiftUI pre builds stuff for development. I also think I had a greater understanding of what I was writing for this project. I think project 1 I was flying by the seat of my pants but this one I was able to understand with much more clarity how things connected. The animals swift example was super helpful for me too. I think having projects like that that we study in class or on our own is super helpful. I think it was hard for me to find valuable questions to ask in a classroom setting. I appriciated the time that was given to ask questions in class but I don't feel that my questions were easy to ask or answer in a classroom setting. AI was great at answering most of these questions. I feel like repalcing some of that QnA time in class with demos of a technique or aspect of the project would have been much more benificial. I did some things that didn't match the example that was given, especailly my editing solution was heavily reliant on holding data in the view. I know that we had a classroom discusison on this but I had already made so much progress on it by that point that I didn't have the time to refactor all of the code to match it. </t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
final updates to the excel spreadsheet before turning it in
</commit_message>
<xml_diff>
--- a/Project 2 Rubric Recipe App.xlsx
+++ b/Project 2 Rubric Recipe App.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/davissl_byu_edu/Documents/BYU/Fall 25/IS 543/Larson Davis Project 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBA1693D-5A96-B044-8F1E-CB661F555780}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="8_{14A3A9A2-8A9D-C34D-9471-868E4F2CDD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C57445E6-4941-174A-8659-323194B973D0}"/>
   <bookViews>
-    <workbookView xWindow="32600" yWindow="-9340" windowWidth="30240" windowHeight="17680" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
+    <workbookView xWindow="38300" yWindow="-9340" windowWidth="30240" windowHeight="17680" xr2:uid="{055AD38E-7EB4-7E46-B9E0-31777D3AA885}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -150,10 +150,10 @@
     <t>N</t>
   </si>
   <si>
-    <t>I tried to add searching by difficulty level but was having issues. After some reasearch I learned that there were some limitations with using #Prediecate in the  FetchDescriptorand an enum to filter. I decided to take it out because it wasn't a requirement and it was taking too much time but it seemed like a simple thing but for the life of me I couldn't get it to work. Another issue that I was having a little difficulty with was handling editing mode in all the nested views. In the category list view there is certain way to edit the categories (by swiping on the category).I was having trouble making the built in edit button give an option to edit the recipe, or make it so that when a user is in edit mode it brings up the edit view when they tap on the recipe. I was getting the nested views mixed up and it was making it hard to get the UI to move to editing like I wanted. I got it to work by removing the edit button itself and add a swipe action but I would say that it is not as understandable as it could be getting to editing views of the reciepes or categories. I think after a little bit of time using the app it becomes understandable but it is not super clear up front.</t>
-  </si>
-  <si>
     <t xml:space="preserve">I enjoyed this project. It was even an app that is useful and practical for my life. It was also cool to see how much swiftUI pre builds stuff for development. I also think I had a greater understanding of what I was writing for this project. I think project 1 I was flying by the seat of my pants but this one I was able to understand with much more clarity how things connected. The animals swift example was super helpful for me too. I think having projects like that that we study in class or on our own is super helpful. I think it was hard for me to find valuable questions to ask in a classroom setting. I appriciated the time that was given to ask questions in class but I don't feel that my questions were easy to ask or answer in a classroom setting. AI was great at answering most of these questions. I feel like repalcing some of that QnA time in class with demos of a technique or aspect of the project would have been much more benificial. I did some things that didn't match the example that was given, especailly my editing solution was heavily reliant on holding data in the view. I know that we had a classroom discusison on this but I had already made so much progress on it by that point that I didn't have the time to refactor all of the code to match it. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">I tried to add searching by difficulty level but was having issues. After some reasearch I learned that there were some limitations with using #Prediecate in the  FetchDescriptorand an enum to filter. I decided to take it out because it wasn't a requirement and it was taking too much time but it seemed like a simple thing but for the life of me I couldn't get it to work. Another issue that I was having a little difficulty with was handling editing mode in all the nested views. In the category list view there is certain way to edit the categories (by swiping on the category).I was having trouble making the built in edit button give an option to edit the recipe, or make it so that when a user is in edit mode it brings up the edit view when they tap on the recipe. I was getting the nested views mixed up and it was making it hard to get the UI to move to editing like I wanted. I got it to work by removing the edit button itself and add a swipe action but I would say that it is not as understandable as it could be getting to editing views of the reciepes or categories. I think after a little bit of time using the app it becomes understandable but it is not super clear up front. </t>
   </si>
 </sst>
 </file>
@@ -753,119 +753,119 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1221,37 +1221,37 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="29"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="44"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
     </row>
     <row r="4" spans="2:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
     </row>
     <row r="6" spans="2:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="59" t="s">
+      <c r="B6" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="59"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
-      <c r="F6" s="59"/>
-      <c r="G6" s="59"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="60"/>
       <c r="H6" s="15" t="s">
         <v>2</v>
       </c>
@@ -1260,46 +1260,43 @@
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="61"/>
       <c r="H7" s="17">
         <v>2</v>
       </c>
       <c r="I7" s="5">
         <v>2</v>
       </c>
-      <c r="J7" s="18">
-        <f>SUM(H7:H26)</f>
-        <v>35</v>
-      </c>
+      <c r="J7" s="18"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
       <c r="H8" s="16"/>
       <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="61"/>
       <c r="H9" s="17">
         <v>2</v>
       </c>
@@ -1308,14 +1305,14 @@
       </c>
     </row>
     <row r="10" spans="2:10" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
       <c r="H10" s="17">
         <v>4</v>
       </c>
@@ -1324,14 +1321,14 @@
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
       <c r="H11" s="17">
         <v>2</v>
       </c>
@@ -1340,14 +1337,14 @@
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="49"/>
       <c r="H12" s="17">
         <v>2</v>
       </c>
@@ -1356,14 +1353,14 @@
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="49"/>
       <c r="H13" s="17">
         <v>2</v>
       </c>
@@ -1373,14 +1370,14 @@
       <c r="J13" s="18"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
+      <c r="C14" s="59"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
+      <c r="G14" s="59"/>
       <c r="H14" s="17">
         <v>2</v>
       </c>
@@ -1390,14 +1387,14 @@
       <c r="J14" s="18"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
+      <c r="C15" s="59"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="59"/>
+      <c r="G15" s="59"/>
       <c r="H15" s="17">
         <v>2</v>
       </c>
@@ -1406,14 +1403,14 @@
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
+      <c r="C16" s="59"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="59"/>
+      <c r="G16" s="59"/>
       <c r="H16" s="17">
         <v>2</v>
       </c>
@@ -1423,14 +1420,14 @@
       <c r="J16" s="18"/>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="59"/>
+      <c r="G17" s="59"/>
       <c r="H17" s="17">
         <v>2</v>
       </c>
@@ -1439,14 +1436,14 @@
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="59"/>
+      <c r="F18" s="59"/>
+      <c r="G18" s="59"/>
       <c r="H18" s="17">
         <v>2</v>
       </c>
@@ -1455,14 +1452,14 @@
       </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="60"/>
-      <c r="D19" s="60"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="60"/>
-      <c r="G19" s="60"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
       <c r="H19" s="9">
         <v>2</v>
       </c>
@@ -1471,14 +1468,14 @@
       </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
+      <c r="C20" s="59"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
       <c r="H20" s="8">
         <v>2</v>
       </c>
@@ -1487,14 +1484,14 @@
       </c>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="59"/>
+      <c r="G21" s="59"/>
       <c r="H21" s="8">
         <v>2</v>
       </c>
@@ -1503,14 +1500,14 @@
       </c>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B22" s="56" t="s">
+      <c r="B22" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="57"/>
-      <c r="D22" s="57"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="58"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="27"/>
       <c r="H22" s="8">
         <v>1</v>
       </c>
@@ -1519,14 +1516,14 @@
       </c>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B23" s="56" t="s">
+      <c r="B23" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="57"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="57"/>
-      <c r="G23" s="58"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="27"/>
       <c r="H23" s="8">
         <v>1</v>
       </c>
@@ -1535,14 +1532,14 @@
       </c>
     </row>
     <row r="24" spans="2:10" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="56" t="s">
+      <c r="B24" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="57"/>
-      <c r="D24" s="57"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="57"/>
-      <c r="G24" s="58"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="27"/>
       <c r="H24" s="8">
         <v>1</v>
       </c>
@@ -1551,14 +1548,14 @@
       </c>
     </row>
     <row r="25" spans="2:10" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="50" t="s">
+      <c r="B25" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="51"/>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="52"/>
+      <c r="C25" s="54"/>
+      <c r="D25" s="54"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="55"/>
       <c r="H25" s="3">
         <v>1</v>
       </c>
@@ -1567,14 +1564,14 @@
       </c>
     </row>
     <row r="26" spans="2:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="53" t="s">
+      <c r="B26" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="55"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="58"/>
       <c r="H26" s="3">
         <v>1</v>
       </c>
@@ -1583,14 +1580,14 @@
       </c>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B27" s="47" t="s">
+      <c r="B27" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="49"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="52"/>
       <c r="H27" s="6" t="s">
         <v>10</v>
       </c>
@@ -1599,24 +1596,24 @@
       </c>
     </row>
     <row r="28" spans="2:10" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="44"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="45"/>
-      <c r="G28" s="46"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="41"/>
       <c r="H28" s="11"/>
       <c r="I28" s="10"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="43"/>
+      <c r="C29" s="45"/>
+      <c r="D29" s="45"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="45"/>
+      <c r="G29" s="48"/>
       <c r="H29" s="6" t="s">
         <v>5</v>
       </c>
@@ -1628,12 +1625,12 @@
       </c>
     </row>
     <row r="30" spans="2:10" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="44"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
-      <c r="G30" s="46"/>
+      <c r="B30" s="39"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="41"/>
       <c r="H30" s="12"/>
       <c r="I30" s="10"/>
       <c r="J30" s="23"/>
@@ -1657,162 +1654,169 @@
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="2:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
     </row>
     <row r="35" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="32" t="s">
+      <c r="B35" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="32"/>
-      <c r="I35" s="32"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="29"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="33" t="s">
+      <c r="B36" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="31"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="32"/>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B37" s="33"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
+      <c r="G37" s="34"/>
+      <c r="H37" s="34"/>
+      <c r="I37" s="35"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B38" s="33"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="34"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
+      <c r="H38" s="34"/>
+      <c r="I38" s="35"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B39" s="33"/>
+      <c r="C39" s="34"/>
+      <c r="D39" s="34"/>
+      <c r="E39" s="34"/>
+      <c r="F39" s="34"/>
+      <c r="G39" s="34"/>
+      <c r="H39" s="34"/>
+      <c r="I39" s="35"/>
+    </row>
+    <row r="40" spans="2:9" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B40" s="36"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="37"/>
+      <c r="E40" s="37"/>
+      <c r="F40" s="37"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="37"/>
+      <c r="I40" s="38"/>
+    </row>
+    <row r="41" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B41" s="24"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="24"/>
+      <c r="G41" s="24"/>
+      <c r="H41" s="24"/>
+      <c r="I41" s="24"/>
+    </row>
+    <row r="43" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B43" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="29"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B44" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="34"/>
-      <c r="F36" s="34"/>
-      <c r="G36" s="34"/>
-      <c r="H36" s="34"/>
-      <c r="I36" s="35"/>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B37" s="36"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="37"/>
-      <c r="I37" s="38"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B38" s="36"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="37"/>
-      <c r="F38" s="37"/>
-      <c r="G38" s="37"/>
-      <c r="H38" s="37"/>
-      <c r="I38" s="38"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B39" s="36"/>
-      <c r="C39" s="37"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="37"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="37"/>
-      <c r="H39" s="37"/>
-      <c r="I39" s="38"/>
-    </row>
-    <row r="40" spans="2:9" ht="121" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="39"/>
-      <c r="C40" s="40"/>
-      <c r="D40" s="40"/>
-      <c r="E40" s="40"/>
-      <c r="F40" s="40"/>
-      <c r="G40" s="40"/>
-      <c r="H40" s="40"/>
-      <c r="I40" s="41"/>
-    </row>
-    <row r="41" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="61"/>
-      <c r="C41" s="61"/>
-      <c r="D41" s="61"/>
-      <c r="E41" s="61"/>
-      <c r="F41" s="61"/>
-      <c r="G41" s="61"/>
-      <c r="H41" s="61"/>
-      <c r="I41" s="61"/>
-    </row>
-    <row r="43" spans="2:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="32"/>
-      <c r="D43" s="32"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="32"/>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B44" s="33" t="s">
-        <v>37</v>
-      </c>
-      <c r="C44" s="34"/>
-      <c r="D44" s="34"/>
-      <c r="E44" s="34"/>
-      <c r="F44" s="34"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="34"/>
-      <c r="I44" s="35"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
+      <c r="E44" s="31"/>
+      <c r="F44" s="31"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="31"/>
+      <c r="I44" s="32"/>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B45" s="36"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="37"/>
-      <c r="F45" s="37"/>
-      <c r="G45" s="37"/>
-      <c r="H45" s="37"/>
-      <c r="I45" s="38"/>
+      <c r="B45" s="33"/>
+      <c r="C45" s="34"/>
+      <c r="D45" s="34"/>
+      <c r="E45" s="34"/>
+      <c r="F45" s="34"/>
+      <c r="G45" s="34"/>
+      <c r="H45" s="34"/>
+      <c r="I45" s="35"/>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B46" s="36"/>
-      <c r="C46" s="37"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="37"/>
-      <c r="F46" s="37"/>
-      <c r="G46" s="37"/>
-      <c r="H46" s="37"/>
-      <c r="I46" s="38"/>
+      <c r="B46" s="33"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+      <c r="E46" s="34"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="34"/>
+      <c r="H46" s="34"/>
+      <c r="I46" s="35"/>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B47" s="36"/>
-      <c r="C47" s="37"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="37"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="37"/>
-      <c r="H47" s="37"/>
-      <c r="I47" s="38"/>
+      <c r="B47" s="33"/>
+      <c r="C47" s="34"/>
+      <c r="D47" s="34"/>
+      <c r="E47" s="34"/>
+      <c r="F47" s="34"/>
+      <c r="G47" s="34"/>
+      <c r="H47" s="34"/>
+      <c r="I47" s="35"/>
     </row>
     <row r="48" spans="2:9" ht="117" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="39"/>
-      <c r="C48" s="40"/>
-      <c r="D48" s="40"/>
-      <c r="E48" s="40"/>
-      <c r="F48" s="40"/>
-      <c r="G48" s="40"/>
-      <c r="H48" s="40"/>
-      <c r="I48" s="41"/>
+      <c r="B48" s="36"/>
+      <c r="C48" s="37"/>
+      <c r="D48" s="37"/>
+      <c r="E48" s="37"/>
+      <c r="F48" s="37"/>
+      <c r="G48" s="37"/>
+      <c r="H48" s="37"/>
+      <c r="I48" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B44:I48"/>
-    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B18:G18"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="B4:I4"/>
@@ -1829,18 +1833,11 @@
     <mergeCell ref="B23:G23"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B14:G14"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B44:I48"/>
+    <mergeCell ref="B30:G30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>